<commit_message>
an analytics tool and backup extension
</commit_message>
<xml_diff>
--- a/variants.xlsx
+++ b/variants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\projects\python\pythonscripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4088EEF-6270-475B-9FCA-582CC9B34B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DE5687-3A2C-4EFE-B466-F80C6078BEE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,222 +33,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>person_uuid</t>
   </si>
   <si>
-    <t>004f2431-f1ec-4e53-883e-3e9daafc4e02</t>
-  </si>
-  <si>
-    <t>019f66e1-badb-4c47-afb1-a2253ca84684</t>
-  </si>
-  <si>
-    <t>04f1fdc9-6c1a-4ca8-a08c-5ddb6f39b5bf</t>
-  </si>
-  <si>
-    <t>068e8593-5d91-44e2-a2cf-23d660d38931</t>
-  </si>
-  <si>
-    <t>0b680895-3ec3-40f1-8da9-63f97421202a</t>
-  </si>
-  <si>
-    <t>0c1b6771-c918-4b39-8e7f-c985c8c0d775</t>
-  </si>
-  <si>
-    <t>0d9cccd4-ebc7-4bc4-9d0d-0e7051bc77dc</t>
-  </si>
-  <si>
-    <t>0e9b1868-d9c2-4878-b22d-423a524c02bd</t>
-  </si>
-  <si>
-    <t>12e824f3-3851-4ec2-8af0-e9374956fe33</t>
-  </si>
-  <si>
-    <t>16618215-c3ee-4707-8d49-f8a181ed542b</t>
-  </si>
-  <si>
-    <t>191c146a-95b0-4a28-8833-9d53df9a7751</t>
-  </si>
-  <si>
-    <t>24e8aa1e-3249-4bb8-a472-ed87d062966c</t>
-  </si>
-  <si>
-    <t>2688f125-dd27-4180-a190-7cb6be6ebce2</t>
-  </si>
-  <si>
-    <t>275eab37-39fd-4036-a384-8a3ee11d0ce3</t>
-  </si>
-  <si>
-    <t>28d44866-c236-4898-a2d2-8bba8102533a</t>
-  </si>
-  <si>
-    <t>29252e33-3ee9-4a42-ac5d-c6cea213eb8e</t>
-  </si>
-  <si>
-    <t>2b0849c4-46e4-4f89-95fc-4fc6f7ccf3d9</t>
-  </si>
-  <si>
-    <t>2cd1765f-f5e2-4283-8340-07fd5e27220c</t>
-  </si>
-  <si>
-    <t>38e418fa-0514-4031-a911-9e26bf4fcefd</t>
-  </si>
-  <si>
-    <t>39a72772-d111-4372-bf3e-d5916771771c</t>
-  </si>
-  <si>
-    <t>3a85a009-322d-4768-bc70-c699e56e41d6</t>
-  </si>
-  <si>
-    <t>4b942f64-8822-47ae-807a-739ee2e396b4</t>
-  </si>
-  <si>
-    <t>4e6080a2-8a17-4704-a8d6-41d7fccbcd52</t>
-  </si>
-  <si>
-    <t>4f7a5545-5c86-4e67-a750-b5e57c1fc04d</t>
-  </si>
-  <si>
-    <t>53c4b258-1ce2-4a69-a93a-99ec13d5d777</t>
-  </si>
-  <si>
-    <t>547d15db-1ac1-4427-9648-701ab2b4b43c</t>
-  </si>
-  <si>
-    <t>61e9dd4d-e5f2-4000-af84-4f9e61bdb412</t>
-  </si>
-  <si>
-    <t>67e447a9-7ab5-49fa-8391-782d62c3ab34</t>
-  </si>
-  <si>
-    <t>6a0d7185-2698-479c-afa6-13c3a5ceab74</t>
-  </si>
-  <si>
-    <t>6c825e25-cab8-4e95-92cb-1efb2661d05b</t>
-  </si>
-  <si>
-    <t>6ca88386-ab46-44d5-a5a4-5464c824115d</t>
-  </si>
-  <si>
-    <t>6d294bee-1dac-4b44-8eef-7aa1f0fe6ea3</t>
-  </si>
-  <si>
-    <t>790a6713-72dc-4771-bdba-475267297495</t>
-  </si>
-  <si>
-    <t>7a09f2e0-19a2-4f57-b3ff-ba127112f511</t>
-  </si>
-  <si>
-    <t>7fae6dd8-9194-4c5d-93dc-56de1680478b</t>
-  </si>
-  <si>
-    <t>89267025-cae2-419d-b1a7-a78391698ac4</t>
-  </si>
-  <si>
-    <t>8bbdae21-2af4-4609-b49c-cb04915d6b7b</t>
-  </si>
-  <si>
-    <t>900b4c26-31f5-41b2-be15-f6c84d6afacd</t>
-  </si>
-  <si>
-    <t>91413f9a-89a6-4962-baee-746a9820e67b</t>
-  </si>
-  <si>
-    <t>94170ac7-5a27-4dba-9a9c-1c6a4135add3</t>
-  </si>
-  <si>
-    <t>9a1050c7-73f8-420e-8e8c-6ace7d792200</t>
-  </si>
-  <si>
-    <t>9d4b4c55-8959-437a-9959-433a262e77c1</t>
-  </si>
-  <si>
-    <t>9e087b06-2770-42e6-b53c-b805fecd96d1</t>
-  </si>
-  <si>
-    <t>9e0d6757-6591-4ba3-a4b3-dada908b4295</t>
-  </si>
-  <si>
-    <t>a0ba8dd4-9322-45cd-b49a-2777612f27cd</t>
-  </si>
-  <si>
-    <t>ae4982a3-ca2a-4fd7-8aba-3f22f5f6129b</t>
-  </si>
-  <si>
-    <t>b418444d-3f9b-42fb-b28a-6da7486fc9e7</t>
-  </si>
-  <si>
-    <t>bd6c0a1b-2378-4467-ac3e-8e61b91e65ef</t>
-  </si>
-  <si>
-    <t>c0206a37-4be8-4a1a-a55c-4b101af20217</t>
-  </si>
-  <si>
-    <t>ca9a1910-6898-4fcd-9ef7-e3b9790ae5c9</t>
-  </si>
-  <si>
-    <t>cc3effe3-60b6-498a-b509-53673584c255</t>
-  </si>
-  <si>
-    <t>cc63628c-cc89-4f98-aa6b-9709337367b7</t>
-  </si>
-  <si>
-    <t>ce89544e-95b7-443f-9bb6-563fcb794ac9</t>
-  </si>
-  <si>
-    <t>cfb0e789-0da8-4737-8311-33babd14dd45</t>
-  </si>
-  <si>
-    <t>d082cf9f-90dd-48c7-b490-d5b228cbaeaa</t>
-  </si>
-  <si>
-    <t>d0b15c90-5d39-4c16-9216-4fcd2d575f2a</t>
-  </si>
-  <si>
-    <t>d23d9ad7-7b40-4f26-8ea6-857a2805ff68</t>
-  </si>
-  <si>
-    <t>d46a2e32-c9ee-49ac-b357-71b29a2b271c</t>
-  </si>
-  <si>
-    <t>d6f5d83f-2591-4e4c-b76e-6a16439d7f23</t>
-  </si>
-  <si>
-    <t>d7bf7d64-1f0a-43d4-9bab-fc974bd42e87</t>
-  </si>
-  <si>
-    <t>dd22c285-c977-43d9-9ace-f9268c271f6e</t>
-  </si>
-  <si>
-    <t>df0a22e1-4839-4f6c-869d-147718100b87</t>
-  </si>
-  <si>
-    <t>e0e37f02-7f30-4786-a4b5-ec406736984f</t>
-  </si>
-  <si>
-    <t>e18125e9-0ca1-44ce-8f68-bb5bdb7a5161</t>
-  </si>
-  <si>
-    <t>e93c802a-3b5a-45bc-bad6-60d05ae32e65</t>
-  </si>
-  <si>
-    <t>ef63c996-f32b-4cb5-8cce-d56300b3ebc2</t>
-  </si>
-  <si>
-    <t>efc61912-158f-4107-9de0-eb0404c52393</t>
-  </si>
-  <si>
-    <t>f257f2f4-d675-42e8-914d-98e3bb3dc30d</t>
-  </si>
-  <si>
-    <t>f8db5dc5-e918-4422-bda2-c7bf68ba94fd</t>
-  </si>
-  <si>
-    <t>f92cd0f0-6754-457a-b69f-77452f338a14</t>
-  </si>
-  <si>
-    <t>fe7e5c0c-2b63-4c90-8745-1c693d978e59</t>
+    <t>fe8f8a87-0362-427e-bd74-095ba668e182</t>
+  </si>
+  <si>
+    <t>cde19b38-d6ec-49a1-9507-de7fd9bc1220</t>
+  </si>
+  <si>
+    <t>d23b3e0e-d716-45f8-a192-11db22649248</t>
+  </si>
+  <si>
+    <t>89137da9-b0fd-4a84-9643-6a8b17f2fc45</t>
+  </si>
+  <si>
+    <t>e8402740-4046-451b-adac-20f4b6d7d7dd</t>
+  </si>
+  <si>
+    <t>ca7247bd-8cd9-48bf-8fbb-caca8e8c4710</t>
+  </si>
+  <si>
+    <t>f73d6e81-0225-4da3-8d40-51fda49620bb</t>
+  </si>
+  <si>
+    <t>a66eafae-fc11-4ca1-a4d3-b39c73d55885</t>
   </si>
 </sst>
 </file>
@@ -277,7 +88,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -288,6 +99,12 @@
       <patternFill patternType="mediumGray">
         <fgColor indexed="9"/>
         <bgColor indexed="54"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -318,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -326,6 +143,7 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -640,359 +458,233 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A10" s="2"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="A11" s="2"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A12" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="A12" s="2"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="A13" s="2"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A14" s="2"/>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A15" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="A15" s="2"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A16" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A16" s="2"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A17" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="A17" s="2"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A18" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="A18" s="2"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A19" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A19" s="2"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A20" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="A20" s="2"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A21" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="A21" s="2"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A22" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A22" s="2"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A23" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A23" s="2"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A24" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A24" s="2"/>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A25" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A25" s="2"/>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A26" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A26" s="2"/>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A27" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A27" s="2"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A28" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="A28" s="2"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A29" s="2" t="s">
-        <v>28</v>
-      </c>
+      <c r="A29" s="2"/>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A30" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="A30" s="2"/>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A31" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="A31" s="2"/>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A32" s="2" t="s">
-        <v>31</v>
-      </c>
+      <c r="A32" s="2"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A33" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="A33" s="2"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A34" s="2" t="s">
-        <v>33</v>
-      </c>
+      <c r="A34" s="2"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A35" s="2" t="s">
-        <v>34</v>
-      </c>
+      <c r="A35" s="2"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A36" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="A36" s="2"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A37" s="2" t="s">
-        <v>36</v>
-      </c>
+      <c r="A37" s="2"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A38" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="A38" s="2"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A39" s="2" t="s">
-        <v>38</v>
-      </c>
+      <c r="A39" s="2"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A40" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="A40" s="2"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A41" s="2" t="s">
-        <v>40</v>
-      </c>
+      <c r="A41" s="2"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A42" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="A42" s="2"/>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A43" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="A43" s="2"/>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A44" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A44" s="2"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A45" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="A45" s="2"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A46" s="2" t="s">
-        <v>45</v>
-      </c>
+      <c r="A46" s="2"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A47" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="A47" s="2"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A48" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="A48" s="2"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A49" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A49" s="2"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A50" s="2" t="s">
-        <v>49</v>
-      </c>
+      <c r="A50" s="2"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A51" s="2" t="s">
-        <v>50</v>
-      </c>
+      <c r="A51" s="2"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A52" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="A52" s="2"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A53" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="A53" s="2"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A54" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="A54" s="2"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A55" s="2" t="s">
-        <v>54</v>
-      </c>
+      <c r="A55" s="2"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A56" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="A56" s="2"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A57" s="2" t="s">
-        <v>56</v>
-      </c>
+      <c r="A57" s="2"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A58" s="2" t="s">
-        <v>57</v>
-      </c>
+      <c r="A58" s="2"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A59" s="2" t="s">
-        <v>58</v>
-      </c>
+      <c r="A59" s="2"/>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A60" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="A60" s="2"/>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A61" s="2" t="s">
-        <v>60</v>
-      </c>
+      <c r="A61" s="2"/>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A62" s="2" t="s">
-        <v>61</v>
-      </c>
+      <c r="A62" s="2"/>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A63" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="A63" s="2"/>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A64" s="2" t="s">
-        <v>63</v>
-      </c>
+      <c r="A64" s="2"/>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A65" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="A65" s="2"/>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A66" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="A66" s="2"/>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A67" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="A67" s="2"/>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A68" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="A68" s="2"/>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A69" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="A69" s="2"/>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A70" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="A70" s="2"/>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A71" s="2" t="s">
-        <v>70</v>
-      </c>
+      <c r="A71" s="2"/>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A72" s="2" t="s">
-        <v>71</v>
-      </c>
+      <c r="A72" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>